<commit_message>
feat(mdx): loai bo triet de Career Stage khoi Query 04 va dong bo MDX, Cube SSAS, Excel
</commit_message>
<xml_diff>
--- a/mdx/Bao_Cao_Double_Check_Query_10_11.xlsx
+++ b/mdx/Bao_Cao_Double_Check_Query_10_11.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query 10 - QoQ Top 10 CLB" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query 11 - Sân trên 60k Chỗ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query 04 - Hieu Suat Do Tuoi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query 10 - QoQ Top 10 CLB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query 11 - Sân trên 60k Chỗ" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -98,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -142,6 +143,21 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -509,6 +525,568 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="104" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BÁO CÁO BÀN THẮNG, KIẾN TẠO &amp; SỐ PHÚT THI ĐẤU TRUNG BÌNH THEO ĐỘ TUỔI NĂM 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Nguồn dữ liệu: SSAS Cube [DW Football Transfermarkt] | Chiều: [DIM Player].[Age], Lát cắt: Year 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Độ Tuổi (Age)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Tổng Bàn Thắng (Goals)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Tổng Kiến Tạo (Assists)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Số Phút TB/Trận (Avg Minutes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>40.31</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>47.78</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>42.69</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>127</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>115</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>44.89</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>298</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>266</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>51.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="19" t="n">
+        <v>24</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>447</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>391</v>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>57.07</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>672</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>536</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>59.74</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>26</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>865</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>694</v>
+      </c>
+      <c r="E14" s="20" t="n">
+        <v>62.56</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>838</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>641</v>
+      </c>
+      <c r="E15" s="21" t="n">
+        <v>63.33</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="19" t="n">
+        <v>28</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>948</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>718</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>66.09</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>1008</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>776</v>
+      </c>
+      <c r="E17" s="21" t="n">
+        <v>67.72</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>816</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>582</v>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>65.17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>632</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>471</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>65.28</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>32</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>720</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>561</v>
+      </c>
+      <c r="E20" s="20" t="n">
+        <v>69.87</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>660</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>484</v>
+      </c>
+      <c r="E21" s="21" t="n">
+        <v>69.45</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="19" t="n">
+        <v>34</v>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>543</v>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>403</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>68.92</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>507</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>316</v>
+      </c>
+      <c r="E23" s="21" t="n">
+        <v>66.56</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="19" t="n">
+        <v>36</v>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>222</v>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>198</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <v>68.58</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="17" t="n">
+        <v>37</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>199</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>139</v>
+      </c>
+      <c r="E25" s="21" t="n">
+        <v>66.51000000000001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="19" t="n">
+        <v>38</v>
+      </c>
+      <c r="C26" s="11" t="n">
+        <v>165</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <v>126</v>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>70.28</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="17" t="n">
+        <v>39</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="E27" s="21" t="n">
+        <v>68.84999999999999</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>65.41</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="17" t="n">
+        <v>41</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="E29" s="21" t="n">
+        <v>71.20999999999999</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="19" t="n">
+        <v>42</v>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>73.11</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="17" t="n">
+        <v>43</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" s="21" t="n">
+        <v>80.28</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="19" t="n">
+        <v>44</v>
+      </c>
+      <c r="C32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="20" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="21" t="n">
+        <v>56.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -537,7 +1115,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -900,7 +1477,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -931,7 +1508,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>